<commit_message>
Daily freezer layout export
</commit_message>
<xml_diff>
--- a/cellstocks/exports/grid-roster.xlsx
+++ b/cellstocks/exports/grid-roster.xlsx
@@ -66757,6 +66757,61 @@
           <t xml:space="preserve">G2</t>
         </is>
       </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cell</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+24</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -66769,6 +66824,61 @@
           <t xml:space="preserve">G3</t>
         </is>
       </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cell</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+24</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -66781,6 +66891,61 @@
           <t xml:space="preserve">G4</t>
         </is>
       </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cell</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+24</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -66910,6 +67075,61 @@
           <t xml:space="preserve">H2</t>
         </is>
       </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cell</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -66920,6 +67140,61 @@
       <c r="B391" t="inlineStr">
         <is>
           <t xml:space="preserve">H3</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cell</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
         </is>
       </c>
     </row>
@@ -68127,17 +68402,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-11</t>
+          <t xml:space="preserve">2026-09-15T08:59:29.978Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -68148,33 +68423,23 @@
       <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 H1</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-10</t>
+          <t xml:space="preserve">2026-09-15T08:59:29.978Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -68185,23 +68450,13 @@
       <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 F6</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T13:48:02.210Z</t>
+          <t xml:space="preserve">2026-09-15T08:59:29.978Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -68211,7 +68466,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -68221,14 +68476,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T13:48:02.210Z</t>
+          <t xml:space="preserve">2026-09-15T08:59:01.686Z</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -68238,7 +68493,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -68255,7 +68510,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T04:57:21.749Z</t>
+          <t xml:space="preserve">2026-09-15T08:59:01.686Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -68265,7 +68520,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -68275,14 +68530,14 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T04:57:21.749Z</t>
+          <t xml:space="preserve">2026-09-15T08:59:01.686Z</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -68292,7 +68547,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -68309,12 +68564,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T04:57:19.918Z</t>
+          <t xml:space="preserve">2026-09-11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -68329,24 +68584,34 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 H1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T04:57:19.918Z</t>
+          <t xml:space="preserve">2026-09-10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -68357,13 +68622,23 @@
       <c r="E9" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 F6</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T04:57:16.692Z</t>
+          <t xml:space="preserve">2026-09-09T13:48:02.210Z</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -68373,7 +68648,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -68390,7 +68665,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09T04:57:16.692Z</t>
+          <t xml:space="preserve">2026-09-09T13:48:02.210Z</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -68400,7 +68675,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -68417,17 +68692,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-09T04:57:21.749Z</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -68438,33 +68713,23 @@
       <c r="E12" t="inlineStr">
         <is>
           <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-09T04:57:21.749Z</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -68474,34 +68739,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-09T04:57:19.918Z</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -68512,33 +68767,23 @@
       <c r="E14" t="inlineStr">
         <is>
           <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-09T04:57:19.918Z</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -68548,29 +68793,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-09T04:57:16.692Z</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -68586,28 +68821,18 @@
       <c r="E16" t="inlineStr">
         <is>
           <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 H3</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-09T04:57:16.692Z</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -68622,17 +68847,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 H2</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
@@ -68649,7 +68864,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -68664,7 +68879,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 B3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -68696,12 +68911,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -68733,12 +68948,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -68760,7 +68975,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -68770,12 +68985,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -68797,7 +69012,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -68807,12 +69022,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 H3</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -68844,12 +69059,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 H3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 H2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -68871,7 +69086,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -68881,12 +69096,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 H2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 B3</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -68908,7 +69123,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -68923,7 +69138,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 B3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -68935,17 +69150,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:53:21.794Z</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -68955,24 +69170,34 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:53:21.794Z</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -68983,23 +69208,33 @@
       <c r="E27" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -69009,24 +69244,34 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -69036,24 +69281,34 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 H3</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -69063,24 +69318,34 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 H2</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -69091,13 +69356,23 @@
       <c r="E31" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 B3</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
+          <t xml:space="preserve">2026-09-08T20:53:21.794Z</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -69107,7 +69382,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -69117,14 +69392,14 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
+          <t xml:space="preserve">2026-09-08T20:53:21.794Z</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -69134,7 +69409,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -69151,7 +69426,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T18:36:51.554Z</t>
+          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -69161,7 +69436,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -69178,7 +69453,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T18:36:51.554Z</t>
+          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -69188,7 +69463,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -69198,14 +69473,14 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T11:09:47.786Z</t>
+          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -69215,7 +69490,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -69232,7 +69507,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T11:09:47.786Z</t>
+          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -69242,7 +69517,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -69259,17 +69534,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -69279,34 +69554,24 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 I8</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-08T20:05:13.592Z</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -69316,34 +69581,24 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-08T18:36:51.554Z</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -69354,33 +69609,23 @@
       <c r="E40" t="inlineStr">
         <is>
           <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A6</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-08T18:36:51.554Z</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -69390,34 +69635,24 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A8</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-08T11:09:47.786Z</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -69428,33 +69663,23 @@
       <c r="E42" t="inlineStr">
         <is>
           <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 E6</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-08T11:09:47.786Z</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">added</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -69464,17 +69689,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 E8</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thaw</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
@@ -69491,7 +69706,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -69506,7 +69721,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 B8</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 I8</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -69528,7 +69743,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -69543,7 +69758,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 D5</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -69565,7 +69780,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -69580,7 +69795,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 D3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A6</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -69602,7 +69817,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -69617,7 +69832,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 D4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A8</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -69639,7 +69854,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -69654,7 +69869,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 E6</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -69676,7 +69891,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -69691,7 +69906,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 E8</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -69713,7 +69928,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -69728,7 +69943,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 B8</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -69750,7 +69965,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -69765,7 +69980,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 D5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -69787,7 +70002,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -69802,7 +70017,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 D3</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -69824,7 +70039,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -69839,7 +70054,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 D4</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -70009,7 +70224,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -70024,7 +70239,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -70061,7 +70276,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -70083,7 +70298,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -70098,7 +70313,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -70120,7 +70335,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -70135,7 +70350,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -70172,7 +70387,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -70209,7 +70424,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -70320,7 +70535,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -70342,7 +70557,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -70352,12 +70567,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 I8</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -70379,7 +70594,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -70389,7 +70604,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -70416,7 +70631,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -70426,12 +70641,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A6</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -70453,7 +70668,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -70463,12 +70678,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A8</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -70490,7 +70705,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -70500,12 +70715,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 E6</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -70527,7 +70742,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -70537,12 +70752,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 E8</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -70564,7 +70779,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -70579,7 +70794,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 B8</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 I8</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -70601,7 +70816,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -70616,7 +70831,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 D5</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -70638,7 +70853,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -70653,7 +70868,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 D3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A6</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -70675,7 +70890,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -70690,7 +70905,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 D4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A8</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -70712,7 +70927,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -70727,7 +70942,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 E6</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -70749,7 +70964,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -70764,7 +70979,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 E8</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -70786,7 +71001,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -70801,7 +71016,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 B8</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -70823,7 +71038,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -70838,7 +71053,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 D5</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -70860,7 +71075,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -70875,7 +71090,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 D3</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -70897,7 +71112,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -70912,7 +71127,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 D4</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -71082,7 +71297,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -71097,7 +71312,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -71134,7 +71349,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -71156,7 +71371,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -71171,7 +71386,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -71193,7 +71408,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -71208,7 +71423,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -71245,7 +71460,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -71282,7 +71497,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -71393,7 +71608,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A2</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -71405,17 +71620,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -71425,24 +71640,34 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A1</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -71452,24 +71677,34 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -71480,23 +71715,33 @@
       <c r="E98" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -71507,23 +71752,33 @@
       <c r="E99" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -71533,24 +71788,34 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A3</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">added</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -71560,14 +71825,24 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1 → Rack 1 A4</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
+          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -71577,7 +71852,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -71587,14 +71862,14 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
+          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -71604,7 +71879,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -71614,14 +71889,14 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
+          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -71631,7 +71906,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -71641,14 +71916,14 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
+          <t xml:space="preserve">2026-09-07T15:21:12.672Z</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -71658,7 +71933,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -71668,14 +71943,14 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -71685,7 +71960,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -71695,14 +71970,14 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -71712,7 +71987,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -71722,14 +71997,14 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -71739,7 +72014,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -71749,14 +72024,14 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:40.838Z</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -71766,7 +72041,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -71776,14 +72051,14 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -71793,7 +72068,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -71803,14 +72078,14 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -71820,7 +72095,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -71830,14 +72105,14 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -71847,7 +72122,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -71857,14 +72132,14 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
+          <t xml:space="preserve">2026-09-07T15:20:16.472Z</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -71874,7 +72149,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek atf3 ox rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -71884,14 +72159,14 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -71901,7 +72176,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -71911,14 +72186,14 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -71928,7 +72203,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek atf3 ox rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -71938,14 +72213,14 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -71955,7 +72230,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -71965,14 +72240,14 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:46.171Z</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -71982,7 +72257,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -71992,14 +72267,14 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -72009,7 +72284,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -72019,14 +72294,14 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -72036,7 +72311,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">hek atf3 ox rep3</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -72046,14 +72321,14 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -72063,7 +72338,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -72073,14 +72348,14 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
+          <t xml:space="preserve">2026-09-07T15:19:15.021Z</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -72090,7 +72365,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">hek atf3 ox rep3</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -72100,14 +72375,14 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
+          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -72117,7 +72392,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -72127,14 +72402,14 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
+          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -72144,7 +72419,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -72154,14 +72429,14 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:17:40.188Z</t>
+          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -72171,7 +72446,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -72181,14 +72456,14 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:17:40.188Z</t>
+          <t xml:space="preserve">2026-09-07T15:18:48.988Z</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -72198,7 +72473,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -72208,14 +72483,14 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t xml:space="preserve">admin</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:17:40.188Z</t>
+          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -72225,7 +72500,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -72235,32 +72510,194 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t xml:space="preserve">umut</t>
+          <t xml:space="preserve">admin</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07T15:18:16.654Z</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
           <t xml:space="preserve">2026-09-07T15:17:40.188Z</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B130" t="inlineStr">
         <is>
           <t xml:space="preserve">added</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D130" t="inlineStr">
         <is>
           <t xml:space="preserve">unknown device</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
+      <c r="E130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07T15:17:40.188Z</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK gNT</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07T15:17:40.188Z</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK gNT</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">umut</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07T15:17:40.188Z</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK gNT</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
         <is>
           <t xml:space="preserve">umut</t>
         </is>

</xml_diff>